<commit_message>
add project title and description minLength
</commit_message>
<xml_diff>
--- a/tests/resources/EVA_Submission_test_V2.xlsx
+++ b/tests/resources/EVA_Submission_test_V2.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="7"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="PLEASE READ FIRST" sheetId="1" state="visible" r:id="rId3"/>
@@ -371,7 +371,7 @@
     <t xml:space="preserve">Brokering institution, if the submission is brokered by another institution to the center producing the project</t>
   </si>
   <si>
-    <t xml:space="preserve">Example Project</t>
+    <t xml:space="preserve">Example Project Title</t>
   </si>
   <si>
     <t xml:space="preserve">An example project for demonstration purposes</t>
@@ -2811,37 +2811,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0e2841"/>
+        <a:srgbClr val="0E2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="e8e8e8"/>
+        <a:srgbClr val="E8E8E8"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="e97132"/>
+        <a:srgbClr val="E97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196b24"/>
+        <a:srgbClr val="196B24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0f9ed5"/>
+        <a:srgbClr val="0F9ED5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="a02b93"/>
+        <a:srgbClr val="A02B93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4ea72e"/>
+        <a:srgbClr val="4EA72E"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607d"/>
+        <a:srgbClr val="96607D"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -3046,7 +3046,7 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" s="4" customFormat="true" ht="67.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" s="4" customFormat="true" ht="79.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
         <v>4</v>
       </c>
@@ -3080,7 +3080,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
     </row>
-    <row r="9" s="4" customFormat="true" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="4" customFormat="true" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
         <v>6</v>
       </c>
@@ -3108,7 +3108,7 @@
       </c>
       <c r="B11" s="16"/>
     </row>
-    <row r="12" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
         <v>8</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="19" t="s">
         <v>10</v>
       </c>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="C13" s="21"/>
     </row>
-    <row r="14" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="40.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
         <v>12</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="67.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="79.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
         <v>14</v>
       </c>
@@ -3141,7 +3141,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="83.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="98.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="24" t="s">
         <v>16</v>
       </c>
@@ -3149,7 +3149,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="50.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="59.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="25" t="s">
         <v>18</v>
       </c>
@@ -7981,7 +7981,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>30</v>
       </c>
@@ -8001,7 +8001,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>36</v>
       </c>
@@ -16721,7 +16721,7 @@
       </c>
       <c r="B17" s="44"/>
     </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="34.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="34" t="s">
         <v>47</v>
       </c>
@@ -16929,7 +16929,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="44" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="50.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
         <v>180</v>
       </c>

</xml_diff>